<commit_message>
Implement manual Leave Management (Sick/Paid Leave) and updated Excel export color-coding
</commit_message>
<xml_diff>
--- a/data/Monthly_Attendance.xlsx
+++ b/data/Monthly_Attendance.xlsx
@@ -34,13 +34,16 @@
     </font>
     <font>
       <color rgb="003730A3"/>
+      <sz val="9"/>
     </font>
     <font>
       <color rgb="00991B1B"/>
+      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00065F46"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="6">
@@ -99,13 +102,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -472,28 +475,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S4"/>
+  <dimension ref="A1:S5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="15" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="15" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -593,10 +596,10 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="30" customHeight="1">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EM001</t>
+          <t>KF001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -674,9 +677,9 @@
           <t>Absent</t>
         </is>
       </c>
-      <c r="Q2" s="4" t="inlineStr">
-        <is>
-          <t>Present</t>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -686,201 +689,302 @@
       </c>
       <c r="S2" s="4" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>IN: 07:28:19
+OUT: 13:40:13</t>
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="30" customHeight="1">
       <c r="A3" t="inlineStr">
         <is>
-          <t>EM002</t>
+          <t>KF003</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>Vikas Prajapat</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="S3" s="4" t="inlineStr">
+        <is>
+          <t>IN: 07:32:59
+OUT: -</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>KF004</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Parth patni</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="S4" s="4" t="inlineStr">
+        <is>
+          <t>IN: 07:55:35
+OUT: -</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>KF002</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>Ashish Pandey</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Holiday</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>Holiday</t>
-        </is>
-      </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="O3" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="P3" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="Q3" s="4" t="inlineStr">
-        <is>
-          <t>Present</t>
-        </is>
-      </c>
-      <c r="R3" s="2" t="inlineStr">
-        <is>
-          <t>Holiday</t>
-        </is>
-      </c>
-      <c r="S3" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>EM003</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Parth Patani</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Holiday</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>Holiday</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="N4" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="O4" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="P4" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="Q4" s="4" t="inlineStr">
-        <is>
-          <t>Present</t>
-        </is>
-      </c>
-      <c r="R4" s="2" t="inlineStr">
-        <is>
-          <t>Holiday</t>
-        </is>
-      </c>
-      <c r="S4" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>Holiday</t>
+        </is>
+      </c>
+      <c r="S5" s="4" t="inlineStr">
+        <is>
+          <t>IN: 13:53:43
+OUT: -</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement historical monthly attendance export with month/year picker
</commit_message>
<xml_diff>
--- a/data/Monthly_Attendance.xlsx
+++ b/data/Monthly_Attendance.xlsx
@@ -43,7 +43,7 @@
     <font>
       <b val="1"/>
       <color rgb="00065F46"/>
-      <sz val="9"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="6">
@@ -481,22 +481,22 @@
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="15" customWidth="1" min="13" max="13"/>
-    <col width="15" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="15" customWidth="1" min="16" max="16"/>
-    <col width="15" customWidth="1" min="17" max="17"/>
-    <col width="15" customWidth="1" min="18" max="18"/>
-    <col width="15" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -596,7 +596,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="42" customHeight="1">
       <c r="A2" t="inlineStr">
         <is>
           <t>KF001</t>
@@ -667,9 +667,10 @@
           <t>Absent</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
+      <c r="O2" s="4" t="inlineStr">
+        <is>
+          <t>IN: Paid Leave
+OUT: Paid Leave</t>
         </is>
       </c>
       <c r="P2" s="3" t="inlineStr">
@@ -689,12 +690,12 @@
       </c>
       <c r="S2" s="4" t="inlineStr">
         <is>
-          <t>IN: 07:28:19
-OUT: 13:40:13</t>
+          <t>IN: Paid Leave
+OUT: Paid Leave</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
+    <row r="3" ht="42" customHeight="1">
       <c r="A3" t="inlineStr">
         <is>
           <t>KF003</t>
@@ -792,7 +793,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1">
+    <row r="4" ht="42" customHeight="1">
       <c r="A4" t="inlineStr">
         <is>
           <t>KF004</t>
@@ -890,7 +891,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5" ht="42" customHeight="1">
       <c r="A5" t="inlineStr">
         <is>
           <t>KF002</t>
@@ -984,7 +985,7 @@
       <c r="S5" s="4" t="inlineStr">
         <is>
           <t>IN: 13:53:43
-OUT: -</t>
+OUT: 14:24:01</t>
         </is>
       </c>
     </row>

</xml_diff>